<commit_message>
Integrate REFramework flow; cleanup pending
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,199 +1,51 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uipath-my.sharepoint.com/personal/alexandra_veizu_uipath_com/Documents/Documents/Projects/REFrameworkNET5/StudioTemplates/REFramework/contentFiles/any/any/pt2/VisualBasic/Data/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{00D541BD-CB78-4D75-8532-9AD73E8C785E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8C54E24-BA5C-4BF9-8DAB-2778512EC11B}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Settings" sheetId="1" r:id="rId1"/>
-    <sheet name="Constants" sheetId="2" r:id="rId2"/>
-    <sheet name="Assets" sheetId="3" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Constants" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="45">
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Asset</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Description (Assets will always overwrite other config)</t>
-  </si>
-  <si>
-    <t>MaxRetryNumber</t>
-  </si>
-  <si>
-    <t>ExScreenshotsFolderPath</t>
-  </si>
-  <si>
-    <t>Exceptions_Screenshots</t>
-  </si>
-  <si>
-    <t>Where to save exceptions screenshots - can be a full or a relative path.</t>
-  </si>
-  <si>
-    <t>LogMessage_GetTransactionData</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Processing Transaction Number: </t>
-  </si>
-  <si>
-    <t>LogMessage_GetTransactionDataError</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Error getting transaction data for Transaction Number: </t>
-  </si>
-  <si>
-    <t>Static part of logging message. Error retrieving Transaction Data.</t>
-  </si>
-  <si>
-    <t>LogMessage_Success</t>
-  </si>
-  <si>
-    <t>Transaction Successful.</t>
-  </si>
-  <si>
-    <t>LogMessage_BusinessRuleException</t>
-  </si>
-  <si>
-    <t>Business rule exception.</t>
-  </si>
-  <si>
-    <t>LogMessage_ApplicationException</t>
-  </si>
-  <si>
-    <t>System exception.</t>
-  </si>
-  <si>
-    <t>logF_BusinessProcessName</t>
-  </si>
-  <si>
-    <t>Framework</t>
-  </si>
-  <si>
-    <t>Orchestrator queue Name. The value must match with the queue name defined on Orchestrator.</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>Logging field which allows grouping of log data of two or more subprocesses under the same business process name</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>OrchestratorQueueName</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>Must be 0 if working with Orchestrator queues. If &gt; 0, the robot will retry the same transaction which failed with a system exception. Must be an integer value.</t>
-  </si>
-  <si>
-    <t>Static part of logging message. Processed Transaction succesful.</t>
-  </si>
-  <si>
-    <t>Static part of logging message. Processed Transaction failed with business exception.</t>
-  </si>
-  <si>
-    <t>Static part of logging message. Processed Transaction failed with application exception.</t>
-  </si>
-  <si>
-    <t>Static part of logging message. Calling Get Transaction Data.</t>
-  </si>
-  <si>
-    <t>OrchestratorAssetFolder</t>
-  </si>
-  <si>
-    <t>OrchestratorQueueFolder</t>
-  </si>
-  <si>
-    <t>Folder name. The value must match a folder defined in Orchestrator and queue specified as OrchestratorQueueName should be created in this folder. For classic folders leave the value field empty.</t>
-  </si>
-  <si>
-    <t>MaxConsecutiveSystemExceptions</t>
-  </si>
-  <si>
-    <t>ExceptionMessage_ConsecutiveErrors</t>
-  </si>
-  <si>
-    <t>RetryNumberGetTransactionItem</t>
-  </si>
-  <si>
-    <t>RetryNumberSetTransactionStatus</t>
-  </si>
-  <si>
-    <t>Error message in case MaxConsecutiveSystemExceptions number is reached.</t>
-  </si>
-  <si>
-    <t>The number of times Get Transaction Item activity is retried in case of an exception. Must be an integer &gt;= 1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The number of times Set transaction status activity is retried in case of an exception. Must be an integer &gt;= 1. </t>
-  </si>
-  <si>
-    <t>ShouldMarkJobAsFaulted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The number of consecutive system exceptions allowed. If MaxConsecutiveSystemExceptions is reached, the job is stopped. To disable this feature, set the value to 0. </t>
-  </si>
-  <si>
-    <t>Must be TRUE or FALSE. If the value is TRUE and an error occurs in Initialization state or the MaxConsecutiveSystemExceptions is reached, the job is marked as Faulted.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The maximum number of consecutive system exceptions was reached. </t>
-  </si>
-  <si>
-    <t>ProcessABCQueue</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="4">
     <font>
+      <name val="Calibri"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
       <sz val="14"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <family val="3"/>
       <sz val="6"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <family val="3"/>
-      <charset val="128"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -212,29 +64,88 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -534,93 +445,139 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z998"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Z6"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="43.5546875" customWidth="1"/>
-    <col min="2" max="2" width="43" customWidth="1"/>
-    <col min="3" max="3" width="81.44140625" customWidth="1"/>
-    <col min="4" max="26" width="8.6640625" customWidth="1"/>
+    <col width="43.5546875" customWidth="1" min="1" max="1"/>
+    <col width="43" customWidth="1" min="2" max="2"/>
+    <col width="81.44140625" customWidth="1" min="3" max="3"/>
+    <col width="8.6640625" customWidth="1" min="4" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
-      <c r="T1" s="1"/>
-      <c r="U1" s="1"/>
-      <c r="V1" s="1"/>
-      <c r="W1" s="1"/>
-      <c r="X1" s="1"/>
-      <c r="Y1" s="1"/>
-      <c r="Z1" s="1"/>
+    <row r="1" ht="14.25" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+      <c r="M1" s="1" t="n"/>
+      <c r="N1" s="1" t="n"/>
+      <c r="O1" s="1" t="n"/>
+      <c r="P1" s="1" t="n"/>
+      <c r="Q1" s="1" t="n"/>
+      <c r="R1" s="1" t="n"/>
+      <c r="S1" s="1" t="n"/>
+      <c r="T1" s="1" t="n"/>
+      <c r="U1" s="1" t="n"/>
+      <c r="V1" s="1" t="n"/>
+      <c r="W1" s="1" t="n"/>
+      <c r="X1" s="1" t="n"/>
+      <c r="Y1" s="1" t="n"/>
+      <c r="Z1" s="1" t="n"/>
     </row>
-    <row r="2" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>22</v>
+    <row r="2" ht="14.25" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>OrchestratorQueueName</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Lyrebird_Validate</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Lyrebird 10_DP input queue (Lyrebird_Validate). Main argument in_OrchestratorQueueName overrides it; an _IT queue switches Main to test mode.</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="43.2">
-      <c r="A3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="4" t="s">
-        <v>32</v>
+    <row r="3" ht="43.2" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>OrchestratorQueueFolder</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Lyrebird</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Orchestrator folder of the input and output queues (Lyrebird). Used by Get Transaction Item, the loader and the performer; Set Transaction Status uses the item itself.</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="5" spans="1:26" ht="28.8">
-      <c r="A5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>23</v>
+    <row r="4" ht="14.25" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>WishlistQueueName</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Lyrebird_Wishlist</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Lyrebird 10_DP output queue for validated albums (input of 20_PF_Download). Main argument in_WishlistQueueName overrides it.</t>
+        </is>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="5" ht="28.8" customHeight="1"/>
+    <row r="6" ht="14.25" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>logF_BusinessProcessName</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Lyrebird_10_DP</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Logging field which allows grouping of log data of two or more subprocesses under the same business process name</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="14.25" customHeight="1"/>
+    <row r="8" ht="14.25" customHeight="1"/>
+    <row r="9" ht="14.25" customHeight="1"/>
+    <row r="10" ht="14.25" customHeight="1"/>
+    <row r="11" ht="14.25" customHeight="1"/>
+    <row r="12" ht="14.25" customHeight="1"/>
+    <row r="13" ht="14.25" customHeight="1"/>
+    <row r="14" ht="14.25" customHeight="1"/>
+    <row r="15" ht="14.25" customHeight="1"/>
+    <row r="16" ht="14.25" customHeight="1"/>
     <row r="17" ht="14.25" customHeight="1"/>
     <row r="18" ht="14.25" customHeight="1"/>
     <row r="19" ht="14.25" customHeight="1"/>
@@ -1604,208 +1561,283 @@
     <row r="997" ht="14.25" customHeight="1"/>
     <row r="998" ht="14.25" customHeight="1"/>
   </sheetData>
-  <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Z988"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Z17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="41" customWidth="1"/>
-    <col min="2" max="2" width="51" customWidth="1"/>
-    <col min="3" max="3" width="75.44140625" customWidth="1"/>
-    <col min="4" max="26" width="8.6640625" customWidth="1"/>
+    <col width="41" customWidth="1" min="1" max="1"/>
+    <col width="51" customWidth="1" min="2" max="2"/>
+    <col width="75.44140625" customWidth="1" min="3" max="3"/>
+    <col width="8.6640625" customWidth="1" min="4" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="14.25" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+      <c r="M1" s="1" t="n"/>
+      <c r="N1" s="1" t="n"/>
+      <c r="O1" s="1" t="n"/>
+      <c r="P1" s="1" t="n"/>
+      <c r="Q1" s="1" t="n"/>
+      <c r="R1" s="1" t="n"/>
+      <c r="S1" s="1" t="n"/>
+      <c r="T1" s="1" t="n"/>
+      <c r="U1" s="1" t="n"/>
+      <c r="V1" s="1" t="n"/>
+      <c r="W1" s="1" t="n"/>
+      <c r="X1" s="1" t="n"/>
+      <c r="Y1" s="1" t="n"/>
+      <c r="Z1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="28.8" customHeight="1">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MaxRetryNumber</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
-      <c r="T1" s="1"/>
-      <c r="U1" s="1"/>
-      <c r="V1" s="1"/>
-      <c r="W1" s="1"/>
-      <c r="X1" s="1"/>
-      <c r="Y1" s="1"/>
-      <c r="Z1" s="1"/>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Must be 0 if working with Orchestrator queues. If &gt; 0, the robot will retry the same transaction which failed with a system exception. Must be an integer value.</t>
+        </is>
+      </c>
     </row>
-    <row r="2" spans="1:26" ht="28.8">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2">
-        <v>0</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>25</v>
+    <row r="3" ht="43.2" customHeight="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MaxConsecutiveSystemExceptions</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Stop the job after 5 consecutive system exceptions (e.g. Supabase or MusicBrainz down), so an outage does not use up the Orchestrator retries of every item. One item can fail 3 times in a row (queue max retries 2).</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="43.2">
-      <c r="A3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>41</v>
+    <row r="4" ht="14.25" customHeight="1"/>
+    <row r="5" ht="14.25" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ExScreenshotsFolderPath</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Exceptions_Screenshots</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Where to save exceptions screenshots - can be a full or a relative path.</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="5" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" t="s">
-        <v>8</v>
+    <row r="6" ht="14.25" customHeight="1"/>
+    <row r="7" ht="14.25" customHeight="1">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LogMessage_GetTransactionData</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Processing Transaction Number: </t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Static part of logging message. Calling Get Transaction Data.</t>
+        </is>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" t="s">
-        <v>29</v>
+    <row r="8" ht="14.25" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>LogMessage_GetTransactionDataError</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error getting transaction data for Transaction Number: </t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Static part of logging message. Error retrieving Transaction Data.</t>
+        </is>
       </c>
     </row>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" t="s">
-        <v>13</v>
+    <row r="9" ht="14.25" customHeight="1">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>LogMessage_Success</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Transaction Successful.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Static part of logging message. Processed Transaction succesful.</t>
+        </is>
       </c>
     </row>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" t="s">
-        <v>26</v>
+    <row r="10" ht="14.25" customHeight="1">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>LogMessage_BusinessRuleException</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Business rule exception.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Static part of logging message. Processed Transaction failed with business exception.</t>
+        </is>
       </c>
     </row>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" t="s">
-        <v>27</v>
+    <row r="11" ht="14.25" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>LogMessage_ApplicationException</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>System exception.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Static part of logging message. Processed Transaction failed with application exception.</t>
+        </is>
       </c>
     </row>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" t="s">
-        <v>28</v>
+    <row r="12" ht="14.25" customHeight="1">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ExceptionMessage_ConsecutiveErrors</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The maximum number of consecutive system exceptions was reached. </t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Error message in case MaxConsecutiveSystemExceptions number is reached.</t>
+        </is>
       </c>
     </row>
-    <row r="12" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A12" t="s">
-        <v>34</v>
-      </c>
-      <c r="B12" t="s">
-        <v>43</v>
-      </c>
-      <c r="C12" t="s">
-        <v>37</v>
+    <row r="13" ht="14.25" customHeight="1"/>
+    <row r="14" ht="14.25" customHeight="1">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>RetryNumberGetTransactionItem</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>The number of times Get Transaction Item activity is retried in case of an exception. Must be an integer &gt;= 1.</t>
+        </is>
       </c>
     </row>
-    <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="14" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A14" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14">
+    <row r="15" ht="14.25" customHeight="1">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>RetryNumberSetTransactionStatus</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
         <v>2</v>
       </c>
-      <c r="C14" t="s">
-        <v>38</v>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The number of times Set transaction status activity is retried in case of an exception. Must be an integer &gt;= 1. </t>
+        </is>
       </c>
     </row>
-    <row r="15" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A15" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15">
-        <v>2</v>
-      </c>
-      <c r="C15" t="s">
-        <v>39</v>
+    <row r="16" ht="14.25" customHeight="1"/>
+    <row r="17" ht="28.8" customHeight="1">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ShouldMarkJobAsFaulted</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Must be TRUE or FALSE. If the value is TRUE and an error occurs in Initialization state or the MaxConsecutiveSystemExceptions is reached, the job is marked as Faulted.</t>
+        </is>
       </c>
     </row>
-    <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" spans="1:3" ht="28.8">
-      <c r="A17" t="s">
-        <v>40</v>
-      </c>
-      <c r="B17" t="b">
-        <v>0</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="19" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="20" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="21" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="22" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="23" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="24" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="25" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="26" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="27" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="28" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="29" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="30" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="31" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="32" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="18" ht="14.25" customHeight="1"/>
+    <row r="19" ht="14.25" customHeight="1"/>
+    <row r="20" ht="14.25" customHeight="1"/>
+    <row r="21" ht="14.25" customHeight="1"/>
+    <row r="22" ht="14.25" customHeight="1"/>
+    <row r="23" ht="14.25" customHeight="1"/>
+    <row r="24" ht="14.25" customHeight="1"/>
+    <row r="25" ht="14.25" customHeight="1"/>
+    <row r="26" ht="14.25" customHeight="1"/>
+    <row r="27" ht="14.25" customHeight="1"/>
+    <row r="28" ht="14.25" customHeight="1"/>
+    <row r="29" ht="14.25" customHeight="1"/>
+    <row r="30" ht="14.25" customHeight="1"/>
+    <row r="31" ht="14.25" customHeight="1"/>
+    <row r="32" ht="14.25" customHeight="1"/>
     <row r="33" ht="14.25" customHeight="1"/>
     <row r="34" ht="14.25" customHeight="1"/>
     <row r="35" ht="14.25" customHeight="1"/>
@@ -2763,73 +2795,84 @@
     <row r="987" ht="14.25" customHeight="1"/>
     <row r="988" ht="14.25" customHeight="1"/>
   </sheetData>
-  <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Z1000"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Z1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31.88671875" customWidth="1"/>
-    <col min="2" max="2" width="30.109375" customWidth="1"/>
-    <col min="3" max="3" width="60.33203125" customWidth="1"/>
-    <col min="4" max="26" width="65.44140625" customWidth="1"/>
+    <col width="31.88671875" customWidth="1" min="1" max="1"/>
+    <col width="30.109375" customWidth="1" min="2" max="2"/>
+    <col width="60.33203125" customWidth="1" min="3" max="3"/>
+    <col width="65.44140625" customWidth="1" min="4" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
-      <c r="T1" s="1"/>
-      <c r="U1" s="1"/>
-      <c r="V1" s="1"/>
-      <c r="W1" s="1"/>
-      <c r="X1" s="1"/>
-      <c r="Y1" s="1"/>
-      <c r="Z1" s="1"/>
+    <row r="1" ht="14.25" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Asset</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>OrchestratorAssetFolder</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Description (Assets will always overwrite other config)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+      <c r="M1" s="1" t="n"/>
+      <c r="N1" s="1" t="n"/>
+      <c r="O1" s="1" t="n"/>
+      <c r="P1" s="1" t="n"/>
+      <c r="Q1" s="1" t="n"/>
+      <c r="R1" s="1" t="n"/>
+      <c r="S1" s="1" t="n"/>
+      <c r="T1" s="1" t="n"/>
+      <c r="U1" s="1" t="n"/>
+      <c r="V1" s="1" t="n"/>
+      <c r="W1" s="1" t="n"/>
+      <c r="X1" s="1" t="n"/>
+      <c r="Y1" s="1" t="n"/>
+      <c r="Z1" s="1" t="n"/>
     </row>
-    <row r="2" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="3" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="5" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="2" ht="14.25" customHeight="1"/>
+    <row r="3" ht="14.25" customHeight="1"/>
+    <row r="4" ht="14.25" customHeight="1"/>
+    <row r="5" ht="14.25" customHeight="1"/>
+    <row r="6" ht="14.25" customHeight="1"/>
+    <row r="7" ht="14.25" customHeight="1"/>
+    <row r="8" ht="14.25" customHeight="1"/>
+    <row r="9" ht="14.25" customHeight="1"/>
+    <row r="10" ht="14.25" customHeight="1"/>
+    <row r="11" ht="14.25" customHeight="1"/>
+    <row r="12" ht="14.25" customHeight="1"/>
+    <row r="13" ht="14.25" customHeight="1"/>
+    <row r="14" ht="14.25" customHeight="1"/>
+    <row r="15" ht="14.25" customHeight="1"/>
+    <row r="16" ht="14.25" customHeight="1"/>
     <row r="17" ht="14.25" customHeight="1"/>
     <row r="18" ht="14.25" customHeight="1"/>
     <row r="19" ht="14.25" customHeight="1"/>
@@ -3815,7 +3858,6 @@
     <row r="999" ht="14.25" customHeight="1"/>
     <row r="1000" ht="14.25" customHeight="1"/>
   </sheetData>
-  <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Integrate REFramework processing and verify recovery paths
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1572,7 +1572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z17"/>
+  <dimension ref="A1:Z16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="41" customWidth="1" min="1" max="1"/>
@@ -1654,131 +1654,129 @@
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1"/>
-    <row r="5" ht="14.25" customHeight="1">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ExScreenshotsFolderPath</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Exceptions_Screenshots</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Where to save exceptions screenshots - can be a full or a relative path.</t>
+    <row r="5" ht="14.25" customHeight="1"/>
+    <row r="6" ht="14.25" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>LogMessage_GetTransactionData</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Processing Transaction Number: </t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Static part of logging message. Calling Get Transaction Data.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="14.25" customHeight="1"/>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LogMessage_GetTransactionData</t>
+          <t>LogMessage_GetTransactionDataError</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Processing Transaction Number: </t>
+          <t xml:space="preserve">Error getting transaction data for Transaction Number: </t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Static part of logging message. Calling Get Transaction Data.</t>
+          <t>Static part of logging message. Error retrieving Transaction Data.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
       <c r="A8" t="inlineStr">
         <is>
-          <t>LogMessage_GetTransactionDataError</t>
+          <t>LogMessage_Success</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error getting transaction data for Transaction Number: </t>
+          <t>Transaction Successful.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Static part of logging message. Error retrieving Transaction Data.</t>
+          <t>Static part of logging message. Processed Transaction succesful.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LogMessage_Success</t>
+          <t>LogMessage_BusinessRuleException</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Transaction Successful.</t>
+          <t>Business rule exception.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Static part of logging message. Processed Transaction succesful.</t>
+          <t>Static part of logging message. Processed Transaction failed with business exception.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LogMessage_BusinessRuleException</t>
+          <t>LogMessage_ApplicationException</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Business rule exception.</t>
+          <t>System exception.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Static part of logging message. Processed Transaction failed with business exception.</t>
+          <t>Static part of logging message. Processed Transaction failed with application exception.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LogMessage_ApplicationException</t>
+          <t>ExceptionMessage_ConsecutiveErrors</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>System exception.</t>
+          <t xml:space="preserve">The maximum number of consecutive system exceptions was reached. </t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Static part of logging message. Processed Transaction failed with application exception.</t>
+          <t>Error message in case MaxConsecutiveSystemExceptions number is reached.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="14.25" customHeight="1">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>ExceptionMessage_ConsecutiveErrors</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The maximum number of consecutive system exceptions was reached. </t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Error message in case MaxConsecutiveSystemExceptions number is reached.</t>
+    <row r="12" ht="14.25" customHeight="1"/>
+    <row r="13" ht="14.25" customHeight="1">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>RetryNumberGetTransactionItem</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>The number of times Get Transaction Item activity is retried in case of an exception. Must be an integer &gt;= 1.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="14.25" customHeight="1"/>
     <row r="14" ht="14.25" customHeight="1">
       <c r="A14" t="inlineStr">
         <is>
-          <t>RetryNumberGetTransactionItem</t>
+          <t>RetryNumberSetTransactionStatus</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1786,43 +1784,29 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>The number of times Get Transaction Item activity is retried in case of an exception. Must be an integer &gt;= 1.</t>
+          <t xml:space="preserve">The number of times Set transaction status activity is retried in case of an exception. Must be an integer &gt;= 1. </t>
         </is>
       </c>
     </row>
-    <row r="15" ht="14.25" customHeight="1">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>RetryNumberSetTransactionStatus</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>2</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The number of times Set transaction status activity is retried in case of an exception. Must be an integer &gt;= 1. </t>
+    <row r="15" ht="14.25" customHeight="1"/>
+    <row r="16" ht="14.25" customHeight="1">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ShouldMarkJobAsFaulted</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Must be TRUE or FALSE. If the value is TRUE and an error occurs in Initialization state or the MaxConsecutiveSystemExceptions is reached, the job is marked as Faulted.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="14.25" customHeight="1"/>
-    <row r="17" ht="28.8" customHeight="1">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>ShouldMarkJobAsFaulted</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Must be TRUE or FALSE. If the value is TRUE and an error occurs in Initialization state or the MaxConsecutiveSystemExceptions is reached, the job is marked as Faulted.</t>
-        </is>
-      </c>
-    </row>
+    <row r="17" ht="28.8" customHeight="1"/>
     <row r="18" ht="14.25" customHeight="1"/>
     <row r="19" ht="14.25" customHeight="1"/>
     <row r="20" ht="14.25" customHeight="1"/>

</xml_diff>